<commit_message>
Update selected EoM yield curve output
</commit_message>
<xml_diff>
--- a/output_eom/Selected_EoM_Yield_Curve.xlsx
+++ b/output_eom/Selected_EoM_Yield_Curve.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI76"/>
+  <dimension ref="A1:AK76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -508,6 +508,8 @@
     <col width="13" customWidth="1" min="33" max="33"/>
     <col width="13" customWidth="1" min="34" max="34"/>
     <col width="13" customWidth="1" min="35" max="35"/>
+    <col width="13" customWidth="1" min="36" max="36"/>
+    <col width="13" customWidth="1" min="37" max="37"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -550,6 +552,8 @@
       <c r="AG1" s="2" t="n"/>
       <c r="AH1" s="2" t="n"/>
       <c r="AI1" s="2" t="n"/>
+      <c r="AJ1" s="2" t="n"/>
+      <c r="AK1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="n"/>
@@ -587,6 +591,8 @@
       <c r="AG2" s="2" t="n"/>
       <c r="AH2" s="2" t="n"/>
       <c r="AI2" s="2" t="n"/>
+      <c r="AJ2" s="2" t="n"/>
+      <c r="AK2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -628,6 +634,8 @@
       <c r="AG3" s="5" t="n"/>
       <c r="AH3" s="5" t="n"/>
       <c r="AI3" s="5" t="n"/>
+      <c r="AJ3" s="5" t="n"/>
+      <c r="AK3" s="5" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n"/>
@@ -665,6 +673,8 @@
       <c r="AG4" s="2" t="n"/>
       <c r="AH4" s="2" t="n"/>
       <c r="AI4" s="2" t="n"/>
+      <c r="AJ4" s="2" t="n"/>
+      <c r="AK4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -774,6 +784,12 @@
       <c r="AI5" s="7" t="n">
         <v>46234</v>
       </c>
+      <c r="AJ5" s="7" t="n">
+        <v>46265</v>
+      </c>
+      <c r="AK5" s="7" t="n">
+        <v>46293</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -947,6 +963,16 @@
         </is>
       </c>
       <c r="AI6" s="8" t="inlineStr">
+        <is>
+          <t>Spot</t>
+        </is>
+      </c>
+      <c r="AJ6" s="8" t="inlineStr">
+        <is>
+          <t>Spot</t>
+        </is>
+      </c>
+      <c r="AK6" s="8" t="inlineStr">
         <is>
           <t>Spot</t>
         </is>
@@ -992,6 +1018,8 @@
       <c r="AG7" s="8" t="n"/>
       <c r="AH7" s="8" t="n"/>
       <c r="AI7" s="8" t="n"/>
+      <c r="AJ7" s="8" t="n"/>
+      <c r="AK7" s="8" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
@@ -1099,6 +1127,12 @@
       <c r="AI8" s="9" t="n">
         <v>0.067942</v>
       </c>
+      <c r="AJ8" s="9" t="n">
+        <v>0.06479600000000001</v>
+      </c>
+      <c r="AK8" s="9" t="n">
+        <v>0.065479</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
@@ -1206,6 +1240,12 @@
       <c r="AI9" s="9" t="n">
         <v>0.069117</v>
       </c>
+      <c r="AJ9" s="9" t="n">
+        <v>0.065736</v>
+      </c>
+      <c r="AK9" s="9" t="n">
+        <v>0.066971</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -1313,6 +1353,12 @@
       <c r="AI10" s="9" t="n">
         <v>0.07026187561013186</v>
       </c>
+      <c r="AJ10" s="9" t="n">
+        <v>0.06664326884281491</v>
+      </c>
+      <c r="AK10" s="9" t="n">
+        <v>0.06808882127577531</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
@@ -1420,6 +1466,12 @@
       <c r="AI11" s="9" t="n">
         <v>0.07132560498938467</v>
       </c>
+      <c r="AJ11" s="9" t="n">
+        <v>0.06743976896564829</v>
+      </c>
+      <c r="AK11" s="9" t="n">
+        <v>0.0689279454628593</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
@@ -1527,6 +1579,12 @@
       <c r="AI12" s="9" t="n">
         <v>0.0721624470825577</v>
       </c>
+      <c r="AJ12" s="9" t="n">
+        <v>0.06813751643655586</v>
+      </c>
+      <c r="AK12" s="9" t="n">
+        <v>0.06961281379319972</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
@@ -1634,6 +1692,12 @@
       <c r="AI13" s="9" t="n">
         <v>0.07273806664115479</v>
       </c>
+      <c r="AJ13" s="9" t="n">
+        <v>0.06874708585194195</v>
+      </c>
+      <c r="AK13" s="9" t="n">
+        <v>0.07018936858337699</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
@@ -1741,6 +1805,12 @@
       <c r="AI14" s="9" t="n">
         <v>0.07309390990393561</v>
       </c>
+      <c r="AJ14" s="9" t="n">
+        <v>0.06927752482070752</v>
+      </c>
+      <c r="AK14" s="9" t="n">
+        <v>0.07067814826710994</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
@@ -1848,6 +1918,12 @@
       <c r="AI15" s="9" t="n">
         <v>0.07329566589252523</v>
       </c>
+      <c r="AJ15" s="9" t="n">
+        <v>0.06973497594183486</v>
+      </c>
+      <c r="AK15" s="9" t="n">
+        <v>0.07108567387771925</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
@@ -1955,6 +2031,12 @@
       <c r="AI16" s="9" t="n">
         <v>0.07340022131115997</v>
       </c>
+      <c r="AJ16" s="9" t="n">
+        <v>0.07012748224072482</v>
+      </c>
+      <c r="AK16" s="9" t="n">
+        <v>0.07141927841320195</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
@@ -2062,6 +2144,12 @@
       <c r="AI17" s="9" t="n">
         <v>0.07344749588812349</v>
       </c>
+      <c r="AJ17" s="9" t="n">
+        <v>0.07046124785220742</v>
+      </c>
+      <c r="AK17" s="9" t="n">
+        <v>0.07168717351426213</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
@@ -2169,6 +2257,12 @@
       <c r="AI18" s="9" t="n">
         <v>0.07346491470401051</v>
       </c>
+      <c r="AJ18" s="9" t="n">
+        <v>0.07074179059622354</v>
+      </c>
+      <c r="AK18" s="9" t="n">
+        <v>0.07189574791142572</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
@@ -2276,6 +2370,12 @@
       <c r="AI19" s="9" t="n">
         <v>0.07346545666904625</v>
       </c>
+      <c r="AJ19" s="9" t="n">
+        <v>0.0709767512376068</v>
+      </c>
+      <c r="AK19" s="9" t="n">
+        <v>0.07205659263333808</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
@@ -2383,6 +2483,12 @@
       <c r="AI20" s="9" t="n">
         <v>0.07345768143278342</v>
       </c>
+      <c r="AJ20" s="9" t="n">
+        <v>0.071170131519177</v>
+      </c>
+      <c r="AK20" s="9" t="n">
+        <v>0.07217656217041113</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
@@ -2490,6 +2596,12 @@
       <c r="AI21" s="9" t="n">
         <v>0.0734481364531645</v>
       </c>
+      <c r="AJ21" s="9" t="n">
+        <v>0.071328060854861</v>
+      </c>
+      <c r="AK21" s="9" t="n">
+        <v>0.07226339595609277</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
@@ -2597,6 +2709,12 @@
       <c r="AI22" s="9" t="n">
         <v>0.07343764954955545</v>
       </c>
+      <c r="AJ22" s="9" t="n">
+        <v>0.07145743815587502</v>
+      </c>
+      <c r="AK22" s="9" t="n">
+        <v>0.07232250092512138</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
@@ -2704,6 +2822,12 @@
       <c r="AI23" s="9" t="n">
         <v>0.07342732969365851</v>
       </c>
+      <c r="AJ23" s="9" t="n">
+        <v>0.07155916889363767</v>
+      </c>
+      <c r="AK23" s="9" t="n">
+        <v>0.07236344366405456</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
@@ -2811,6 +2935,12 @@
       <c r="AI24" s="9" t="n">
         <v>0.07341674580517021</v>
       </c>
+      <c r="AJ24" s="9" t="n">
+        <v>0.07163974703953713</v>
+      </c>
+      <c r="AK24" s="9" t="n">
+        <v>0.07238797038812406</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
@@ -2918,6 +3048,12 @@
       <c r="AI25" s="9" t="n">
         <v>0.07340740716669591</v>
       </c>
+      <c r="AJ25" s="9" t="n">
+        <v>0.07170275147326688</v>
+      </c>
+      <c r="AK25" s="9" t="n">
+        <v>0.0724018903133945</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
@@ -3025,6 +3161,12 @@
       <c r="AI26" s="9" t="n">
         <v>0.07339910622292467</v>
       </c>
+      <c r="AJ26" s="9" t="n">
+        <v>0.0717503212562014</v>
+      </c>
+      <c r="AK26" s="9" t="n">
+        <v>0.07240784939935074</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n">
@@ -3132,6 +3274,12 @@
       <c r="AI27" s="9" t="n">
         <v>0.07339167911712163</v>
       </c>
+      <c r="AJ27" s="9" t="n">
+        <v>0.07178493672716217</v>
+      </c>
+      <c r="AK27" s="9" t="n">
+        <v>0.07240685662962587</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n">
@@ -3239,6 +3387,12 @@
       <c r="AI28" s="9" t="n">
         <v>0.07338499476583737</v>
       </c>
+      <c r="AJ28" s="9" t="n">
+        <v>0.07180944713373671</v>
+      </c>
+      <c r="AK28" s="9" t="n">
+        <v>0.07240224624256086</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
@@ -3346,6 +3500,12 @@
       <c r="AI29" s="9" t="n">
         <v>0.07337894705530501</v>
       </c>
+      <c r="AJ29" s="9" t="n">
+        <v>0.07182710304335901</v>
+      </c>
+      <c r="AK29" s="9" t="n">
+        <v>0.07239337392483858</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n">
@@ -3453,6 +3613,12 @@
       <c r="AI30" s="9" t="n">
         <v>0.07337344916620792</v>
       </c>
+      <c r="AJ30" s="9" t="n">
+        <v>0.07183699352996531</v>
+      </c>
+      <c r="AK30" s="9" t="n">
+        <v>0.07238421746742429</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n">
@@ -3560,6 +3726,12 @@
       <c r="AI31" s="9" t="n">
         <v>0.07336842937901755</v>
       </c>
+      <c r="AJ31" s="9" t="n">
+        <v>0.07184058981297184</v>
+      </c>
+      <c r="AK31" s="9" t="n">
+        <v>0.07237443294199664</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n">
@@ -3667,6 +3839,12 @@
       <c r="AI32" s="9" t="n">
         <v>0.07336382792804885</v>
       </c>
+      <c r="AJ32" s="9" t="n">
+        <v>0.07183959582845612</v>
+      </c>
+      <c r="AK32" s="9" t="n">
+        <v>0.07236369648576479</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n">
@@ -3774,6 +3952,12 @@
       <c r="AI33" s="9" t="n">
         <v>0.07335959461058006</v>
       </c>
+      <c r="AJ33" s="9" t="n">
+        <v>0.07183596891101951</v>
+      </c>
+      <c r="AK33" s="9" t="n">
+        <v>0.07235169685656051</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n">
@@ -3881,6 +4065,12 @@
       <c r="AI34" s="9" t="n">
         <v>0.07335568694773542</v>
       </c>
+      <c r="AJ34" s="9" t="n">
+        <v>0.0718319437625294</v>
+      </c>
+      <c r="AK34" s="9" t="n">
+        <v>0.07234087962833713</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n">
@@ -3988,6 +4178,12 @@
       <c r="AI35" s="9" t="n">
         <v>0.07335206875408229</v>
       </c>
+      <c r="AJ35" s="9" t="n">
+        <v>0.07182433172590041</v>
+      </c>
+      <c r="AK35" s="9" t="n">
+        <v>0.07233112874170367</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n">
@@ -4095,6 +4291,12 @@
       <c r="AI36" s="9" t="n">
         <v>0.0733487090137539</v>
       </c>
+      <c r="AJ36" s="9" t="n">
+        <v>0.07181561460921496</v>
+      </c>
+      <c r="AK36" s="9" t="n">
+        <v>0.07231933667907686</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n">
@@ -4202,6 +4404,12 @@
       <c r="AI37" s="9" t="n">
         <v>0.07334558098910859</v>
       </c>
+      <c r="AJ37" s="9" t="n">
+        <v>0.0718054694571757</v>
+      </c>
+      <c r="AK37" s="9" t="n">
+        <v>0.07230835797871582</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n">
@@ -4308,6 +4516,12 @@
       </c>
       <c r="AI38" s="9" t="n">
         <v>0.07334266150766444</v>
+      </c>
+      <c r="AJ38" s="9" t="n">
+        <v>0.07179357211579555</v>
+      </c>
+      <c r="AK38" s="9" t="n">
+        <v>0.07230140783380112</v>
       </c>
     </row>
     <row r="39">
@@ -4346,6 +4560,8 @@
       <c r="AG39" s="2" t="n"/>
       <c r="AH39" s="2" t="n"/>
       <c r="AI39" s="2" t="n"/>
+      <c r="AJ39" s="2" t="n"/>
+      <c r="AK39" s="2" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="n"/>
@@ -4383,6 +4599,8 @@
       <c r="AG40" s="2" t="n"/>
       <c r="AH40" s="2" t="n"/>
       <c r="AI40" s="2" t="n"/>
+      <c r="AJ40" s="2" t="n"/>
+      <c r="AK40" s="2" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="n"/>
@@ -4420,6 +4638,8 @@
       <c r="AG41" s="2" t="n"/>
       <c r="AH41" s="2" t="n"/>
       <c r="AI41" s="2" t="n"/>
+      <c r="AJ41" s="2" t="n"/>
+      <c r="AK41" s="2" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -4461,6 +4681,8 @@
       <c r="AG42" s="5" t="n"/>
       <c r="AH42" s="5" t="n"/>
       <c r="AI42" s="5" t="n"/>
+      <c r="AJ42" s="5" t="n"/>
+      <c r="AK42" s="5" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="n"/>
@@ -4498,6 +4720,8 @@
       <c r="AG43" s="2" t="n"/>
       <c r="AH43" s="2" t="n"/>
       <c r="AI43" s="2" t="n"/>
+      <c r="AJ43" s="2" t="n"/>
+      <c r="AK43" s="2" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
@@ -4607,6 +4831,12 @@
       <c r="AI44" s="7" t="n">
         <v>46234</v>
       </c>
+      <c r="AJ44" s="7" t="n">
+        <v>46265</v>
+      </c>
+      <c r="AK44" s="7" t="n">
+        <v>46293</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
@@ -4780,6 +5010,16 @@
         </is>
       </c>
       <c r="AI45" s="8" t="inlineStr">
+        <is>
+          <t>Forward</t>
+        </is>
+      </c>
+      <c r="AJ45" s="8" t="inlineStr">
+        <is>
+          <t>Forward</t>
+        </is>
+      </c>
+      <c r="AK45" s="8" t="inlineStr">
         <is>
           <t>Forward</t>
         </is>
@@ -4825,6 +5065,8 @@
       <c r="AG46" s="8" t="n"/>
       <c r="AH46" s="8" t="n"/>
       <c r="AI46" s="8" t="n"/>
+      <c r="AJ46" s="8" t="n"/>
+      <c r="AK46" s="8" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="3" t="n">
@@ -4966,6 +5208,14 @@
         <f>AI9</f>
         <v/>
       </c>
+      <c r="AJ47" s="9">
+        <f>AJ9</f>
+        <v/>
+      </c>
+      <c r="AK47" s="9">
+        <f>AK9</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n">
@@ -5107,6 +5357,14 @@
         <f>((1+AI10)^$A10/((1+AI9)^$A9))-1</f>
         <v/>
       </c>
+      <c r="AJ48" s="9">
+        <f>((1+AJ10)^$A10/((1+AJ9)^$A9))-1</f>
+        <v/>
+      </c>
+      <c r="AK48" s="9">
+        <f>((1+AK10)^$A10/((1+AK9)^$A9))-1</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="n">
@@ -5248,6 +5506,14 @@
         <f>((1+AI11)^$A11/((1+AI10)^$A10))-1</f>
         <v/>
       </c>
+      <c r="AJ49" s="9">
+        <f>((1+AJ11)^$A11/((1+AJ10)^$A10))-1</f>
+        <v/>
+      </c>
+      <c r="AK49" s="9">
+        <f>((1+AK11)^$A11/((1+AK10)^$A10))-1</f>
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="n">
@@ -5389,6 +5655,14 @@
         <f>((1+AI12)^$A12/((1+AI11)^$A11))-1</f>
         <v/>
       </c>
+      <c r="AJ50" s="9">
+        <f>((1+AJ12)^$A12/((1+AJ11)^$A11))-1</f>
+        <v/>
+      </c>
+      <c r="AK50" s="9">
+        <f>((1+AK12)^$A12/((1+AK11)^$A11))-1</f>
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="n">
@@ -5530,6 +5804,14 @@
         <f>((1+AI13)^$A13/((1+AI12)^$A12))-1</f>
         <v/>
       </c>
+      <c r="AJ51" s="9">
+        <f>((1+AJ13)^$A13/((1+AJ12)^$A12))-1</f>
+        <v/>
+      </c>
+      <c r="AK51" s="9">
+        <f>((1+AK13)^$A13/((1+AK12)^$A12))-1</f>
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="n">
@@ -5671,6 +5953,14 @@
         <f>((1+AI14)^$A14/((1+AI13)^$A13))-1</f>
         <v/>
       </c>
+      <c r="AJ52" s="9">
+        <f>((1+AJ14)^$A14/((1+AJ13)^$A13))-1</f>
+        <v/>
+      </c>
+      <c r="AK52" s="9">
+        <f>((1+AK14)^$A14/((1+AK13)^$A13))-1</f>
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="n">
@@ -5812,6 +6102,14 @@
         <f>((1+AI15)^$A15/((1+AI14)^$A14))-1</f>
         <v/>
       </c>
+      <c r="AJ53" s="9">
+        <f>((1+AJ15)^$A15/((1+AJ14)^$A14))-1</f>
+        <v/>
+      </c>
+      <c r="AK53" s="9">
+        <f>((1+AK15)^$A15/((1+AK14)^$A14))-1</f>
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="n">
@@ -5953,6 +6251,14 @@
         <f>((1+AI16)^$A16/((1+AI15)^$A15))-1</f>
         <v/>
       </c>
+      <c r="AJ54" s="9">
+        <f>((1+AJ16)^$A16/((1+AJ15)^$A15))-1</f>
+        <v/>
+      </c>
+      <c r="AK54" s="9">
+        <f>((1+AK16)^$A16/((1+AK15)^$A15))-1</f>
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="n">
@@ -6094,6 +6400,14 @@
         <f>((1+AI17)^$A17/((1+AI16)^$A16))-1</f>
         <v/>
       </c>
+      <c r="AJ55" s="9">
+        <f>((1+AJ17)^$A17/((1+AJ16)^$A16))-1</f>
+        <v/>
+      </c>
+      <c r="AK55" s="9">
+        <f>((1+AK17)^$A17/((1+AK16)^$A16))-1</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="n">
@@ -6235,6 +6549,14 @@
         <f>((1+AI18)^$A18/((1+AI17)^$A17))-1</f>
         <v/>
       </c>
+      <c r="AJ56" s="9">
+        <f>((1+AJ18)^$A18/((1+AJ17)^$A17))-1</f>
+        <v/>
+      </c>
+      <c r="AK56" s="9">
+        <f>((1+AK18)^$A18/((1+AK17)^$A17))-1</f>
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="n">
@@ -6376,6 +6698,14 @@
         <f>((1+AI19)^$A19/((1+AI18)^$A18))-1</f>
         <v/>
       </c>
+      <c r="AJ57" s="9">
+        <f>((1+AJ19)^$A19/((1+AJ18)^$A18))-1</f>
+        <v/>
+      </c>
+      <c r="AK57" s="9">
+        <f>((1+AK19)^$A19/((1+AK18)^$A18))-1</f>
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="n">
@@ -6517,6 +6847,14 @@
         <f>((1+AI20)^$A20/((1+AI19)^$A19))-1</f>
         <v/>
       </c>
+      <c r="AJ58" s="9">
+        <f>((1+AJ20)^$A20/((1+AJ19)^$A19))-1</f>
+        <v/>
+      </c>
+      <c r="AK58" s="9">
+        <f>((1+AK20)^$A20/((1+AK19)^$A19))-1</f>
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="n">
@@ -6658,6 +6996,14 @@
         <f>((1+AI21)^$A21/((1+AI20)^$A20))-1</f>
         <v/>
       </c>
+      <c r="AJ59" s="9">
+        <f>((1+AJ21)^$A21/((1+AJ20)^$A20))-1</f>
+        <v/>
+      </c>
+      <c r="AK59" s="9">
+        <f>((1+AK21)^$A21/((1+AK20)^$A20))-1</f>
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="n">
@@ -6799,6 +7145,14 @@
         <f>((1+AI22)^$A22/((1+AI21)^$A21))-1</f>
         <v/>
       </c>
+      <c r="AJ60" s="9">
+        <f>((1+AJ22)^$A22/((1+AJ21)^$A21))-1</f>
+        <v/>
+      </c>
+      <c r="AK60" s="9">
+        <f>((1+AK22)^$A22/((1+AK21)^$A21))-1</f>
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="n">
@@ -6940,6 +7294,14 @@
         <f>((1+AI23)^$A23/((1+AI22)^$A22))-1</f>
         <v/>
       </c>
+      <c r="AJ61" s="9">
+        <f>((1+AJ23)^$A23/((1+AJ22)^$A22))-1</f>
+        <v/>
+      </c>
+      <c r="AK61" s="9">
+        <f>((1+AK23)^$A23/((1+AK22)^$A22))-1</f>
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="n">
@@ -7081,6 +7443,14 @@
         <f>((1+AI24)^$A24/((1+AI23)^$A23))-1</f>
         <v/>
       </c>
+      <c r="AJ62" s="9">
+        <f>((1+AJ24)^$A24/((1+AJ23)^$A23))-1</f>
+        <v/>
+      </c>
+      <c r="AK62" s="9">
+        <f>((1+AK24)^$A24/((1+AK23)^$A23))-1</f>
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="n">
@@ -7222,6 +7592,14 @@
         <f>((1+AI25)^$A25/((1+AI24)^$A24))-1</f>
         <v/>
       </c>
+      <c r="AJ63" s="9">
+        <f>((1+AJ25)^$A25/((1+AJ24)^$A24))-1</f>
+        <v/>
+      </c>
+      <c r="AK63" s="9">
+        <f>((1+AK25)^$A25/((1+AK24)^$A24))-1</f>
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="n">
@@ -7363,6 +7741,14 @@
         <f>((1+AI26)^$A26/((1+AI25)^$A25))-1</f>
         <v/>
       </c>
+      <c r="AJ64" s="9">
+        <f>((1+AJ26)^$A26/((1+AJ25)^$A25))-1</f>
+        <v/>
+      </c>
+      <c r="AK64" s="9">
+        <f>((1+AK26)^$A26/((1+AK25)^$A25))-1</f>
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="n">
@@ -7504,6 +7890,14 @@
         <f>((1+AI27)^$A27/((1+AI26)^$A26))-1</f>
         <v/>
       </c>
+      <c r="AJ65" s="9">
+        <f>((1+AJ27)^$A27/((1+AJ26)^$A26))-1</f>
+        <v/>
+      </c>
+      <c r="AK65" s="9">
+        <f>((1+AK27)^$A27/((1+AK26)^$A26))-1</f>
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="n">
@@ -7645,6 +8039,14 @@
         <f>((1+AI28)^$A28/((1+AI27)^$A27))-1</f>
         <v/>
       </c>
+      <c r="AJ66" s="9">
+        <f>((1+AJ28)^$A28/((1+AJ27)^$A27))-1</f>
+        <v/>
+      </c>
+      <c r="AK66" s="9">
+        <f>((1+AK28)^$A28/((1+AK27)^$A27))-1</f>
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="n">
@@ -7786,6 +8188,14 @@
         <f>((1+AI29)^$A29/((1+AI28)^$A28))-1</f>
         <v/>
       </c>
+      <c r="AJ67" s="9">
+        <f>((1+AJ29)^$A29/((1+AJ28)^$A28))-1</f>
+        <v/>
+      </c>
+      <c r="AK67" s="9">
+        <f>((1+AK29)^$A29/((1+AK28)^$A28))-1</f>
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="n">
@@ -7927,6 +8337,14 @@
         <f>((1+AI30)^$A30/((1+AI29)^$A29))-1</f>
         <v/>
       </c>
+      <c r="AJ68" s="9">
+        <f>((1+AJ30)^$A30/((1+AJ29)^$A29))-1</f>
+        <v/>
+      </c>
+      <c r="AK68" s="9">
+        <f>((1+AK30)^$A30/((1+AK29)^$A29))-1</f>
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="n">
@@ -8068,6 +8486,14 @@
         <f>((1+AI31)^$A31/((1+AI30)^$A30))-1</f>
         <v/>
       </c>
+      <c r="AJ69" s="9">
+        <f>((1+AJ31)^$A31/((1+AJ30)^$A30))-1</f>
+        <v/>
+      </c>
+      <c r="AK69" s="9">
+        <f>((1+AK31)^$A31/((1+AK30)^$A30))-1</f>
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="n">
@@ -8209,6 +8635,14 @@
         <f>((1+AI32)^$A32/((1+AI31)^$A31))-1</f>
         <v/>
       </c>
+      <c r="AJ70" s="9">
+        <f>((1+AJ32)^$A32/((1+AJ31)^$A31))-1</f>
+        <v/>
+      </c>
+      <c r="AK70" s="9">
+        <f>((1+AK32)^$A32/((1+AK31)^$A31))-1</f>
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="n">
@@ -8350,6 +8784,14 @@
         <f>((1+AI33)^$A33/((1+AI32)^$A32))-1</f>
         <v/>
       </c>
+      <c r="AJ71" s="9">
+        <f>((1+AJ33)^$A33/((1+AJ32)^$A32))-1</f>
+        <v/>
+      </c>
+      <c r="AK71" s="9">
+        <f>((1+AK33)^$A33/((1+AK32)^$A32))-1</f>
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="n">
@@ -8491,6 +8933,14 @@
         <f>((1+AI34)^$A34/((1+AI33)^$A33))-1</f>
         <v/>
       </c>
+      <c r="AJ72" s="9">
+        <f>((1+AJ34)^$A34/((1+AJ33)^$A33))-1</f>
+        <v/>
+      </c>
+      <c r="AK72" s="9">
+        <f>((1+AK34)^$A34/((1+AK33)^$A33))-1</f>
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="n">
@@ -8632,6 +9082,14 @@
         <f>((1+AI35)^$A35/((1+AI34)^$A34))-1</f>
         <v/>
       </c>
+      <c r="AJ73" s="9">
+        <f>((1+AJ35)^$A35/((1+AJ34)^$A34))-1</f>
+        <v/>
+      </c>
+      <c r="AK73" s="9">
+        <f>((1+AK35)^$A35/((1+AK34)^$A34))-1</f>
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="3" t="n">
@@ -8773,6 +9231,14 @@
         <f>((1+AI36)^$A36/((1+AI35)^$A35))-1</f>
         <v/>
       </c>
+      <c r="AJ74" s="9">
+        <f>((1+AJ36)^$A36/((1+AJ35)^$A35))-1</f>
+        <v/>
+      </c>
+      <c r="AK74" s="9">
+        <f>((1+AK36)^$A36/((1+AK35)^$A35))-1</f>
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="n">
@@ -8914,6 +9380,14 @@
         <f>((1+AI37)^$A37/((1+AI36)^$A36))-1</f>
         <v/>
       </c>
+      <c r="AJ75" s="9">
+        <f>((1+AJ37)^$A37/((1+AJ36)^$A36))-1</f>
+        <v/>
+      </c>
+      <c r="AK75" s="9">
+        <f>((1+AK37)^$A37/((1+AK36)^$A36))-1</f>
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="n">
@@ -9053,6 +9527,14 @@
       </c>
       <c r="AI76" s="9">
         <f>((1+AI38)^$A38/((1+AI37)^$A37))-1</f>
+        <v/>
+      </c>
+      <c r="AJ76" s="9">
+        <f>((1+AJ38)^$A38/((1+AJ37)^$A37))-1</f>
+        <v/>
+      </c>
+      <c r="AK76" s="9">
+        <f>((1+AK38)^$A38/((1+AK37)^$A37))-1</f>
         <v/>
       </c>
     </row>

</xml_diff>